<commit_message>
Zmiany struktury folderów oraz czyszczenie zbędnych plików
</commit_message>
<xml_diff>
--- a/Docs/WiKiModule/Audyt Energetyczny.xlsx
+++ b/Docs/WiKiModule/Audyt Energetyczny.xlsx
@@ -1,20 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bolka\Desktop\Supla Warsztat\Projekty\Regulator PID\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bolka\Documents\PlatformIO\Projects\Regulator-PID-VSC\Docs\WiKiModule\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2EEDB347-92AA-49D0-AEA3-DE1AA971A723}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C6F6AFE0-A132-4A5F-BAB0-7A07FF0CB25A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-103" yWindow="-103" windowWidth="22149" windowHeight="13200" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-103" yWindow="18411" windowWidth="22149" windowHeight="13200" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Arkusz1" sheetId="1" r:id="rId1"/>
-    <sheet name="Arkusz2" sheetId="2" r:id="rId2"/>
+    <sheet name="Moduły" sheetId="1" r:id="rId1"/>
+    <sheet name="Rezystancja" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -440,7 +440,7 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -736,16 +736,16 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:E21"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="14.75" x14ac:dyDescent="0.75"/>
   <cols>
-    <col min="1" max="1" width="27.84375" customWidth="1"/>
-    <col min="2" max="2" width="21.23046875" customWidth="1"/>
-    <col min="3" max="3" width="25.23046875" customWidth="1"/>
-    <col min="4" max="4" width="25.61328125" customWidth="1"/>
-    <col min="5" max="5" width="35.3046875" customWidth="1"/>
+    <col min="1" max="1" width="27.81640625" customWidth="1"/>
+    <col min="2" max="2" width="21.2265625" customWidth="1"/>
+    <col min="3" max="3" width="25.2265625" customWidth="1"/>
+    <col min="4" max="4" width="25.58984375" customWidth="1"/>
+    <col min="5" max="5" width="35.31640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:5" ht="15.5" thickBot="1" x14ac:dyDescent="0.9">
       <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
@@ -762,7 +762,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.75">
       <c r="A2" s="6" t="s">
         <v>5</v>
       </c>
@@ -779,7 +779,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="3" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.75">
       <c r="A3" s="6" t="s">
         <v>10</v>
       </c>
@@ -796,7 +796,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="4" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.75">
       <c r="A4" s="6" t="s">
         <v>15</v>
       </c>
@@ -813,7 +813,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="5" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.75">
       <c r="A5" s="6" t="s">
         <v>20</v>
       </c>
@@ -830,7 +830,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="6" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.75">
       <c r="A6" s="6" t="s">
         <v>24</v>
       </c>
@@ -847,7 +847,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="7" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.75">
       <c r="A7" s="6" t="s">
         <v>27</v>
       </c>
@@ -864,7 +864,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="8" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.75">
       <c r="A8" s="6" t="s">
         <v>31</v>
       </c>
@@ -881,7 +881,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="9" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.75">
       <c r="A9" s="6" t="s">
         <v>34</v>
       </c>
@@ -898,7 +898,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.75">
       <c r="A10" s="6" t="s">
         <v>39</v>
       </c>
@@ -915,7 +915,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="11" spans="1:5" ht="22.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:5" ht="22.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.9">
       <c r="A11" s="7" t="s">
         <v>40</v>
       </c>
@@ -930,7 +930,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="21" spans="5:5" x14ac:dyDescent="0.4">
+    <row r="21" spans="5:5" x14ac:dyDescent="0.75">
       <c r="E21" s="10"/>
     </row>
   </sheetData>
@@ -941,15 +941,15 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{093EA34E-7583-46FC-B955-9A80F9695BBC}">
   <dimension ref="A1:D5"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="14.75" x14ac:dyDescent="0.75"/>
   <cols>
-    <col min="1" max="1" width="34.69140625" customWidth="1"/>
-    <col min="2" max="2" width="31.15234375" customWidth="1"/>
-    <col min="3" max="3" width="43.61328125" customWidth="1"/>
-    <col min="4" max="4" width="44.765625" customWidth="1"/>
+    <col min="1" max="1" width="34.6796875" customWidth="1"/>
+    <col min="2" max="2" width="31.1328125" customWidth="1"/>
+    <col min="3" max="3" width="43.58984375" customWidth="1"/>
+    <col min="4" max="4" width="44.76953125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:4" ht="29.75" thickBot="1" x14ac:dyDescent="0.9">
       <c r="A1" s="14" t="s">
         <v>44</v>
       </c>
@@ -963,7 +963,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:4" ht="29" x14ac:dyDescent="0.75">
       <c r="A2" s="12" t="s">
         <v>48</v>
       </c>
@@ -977,7 +977,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:4" ht="29" x14ac:dyDescent="0.75">
       <c r="A3" s="12" t="s">
         <v>51</v>
       </c>
@@ -991,7 +991,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.75">
       <c r="A4" s="12" t="s">
         <v>54</v>
       </c>
@@ -1005,7 +1005,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="5" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:4" ht="29.25" thickBot="1" x14ac:dyDescent="0.9">
       <c r="A5" s="13" t="s">
         <v>57</v>
       </c>

</xml_diff>